<commit_message>
Added E2E flow on Creative Bulk upload. And modified new methods to incorporate bulk upload changes
</commit_message>
<xml_diff>
--- a/src/main/resources/uploadfiles/DCM_HTML_BulkUpload.xlsx
+++ b/src/main/resources/uploadfiles/DCM_HTML_BulkUpload.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rsherkar\IdeaProjects\PulsePointNew\src\main\resources\uploadfiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03BB2202-A2EF-474E-880A-45E7BABBF357}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F0161CF-B862-40F5-8F68-E2ACC4CE2CDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="374" xr2:uid="{386F8AE9-53F9-4036-A21A-50DAAB348328}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="374" activeTab="1" xr2:uid="{386F8AE9-53F9-4036-A21A-50DAAB348328}"/>
   </bookViews>
   <sheets>
     <sheet name="Tags" sheetId="1" r:id="rId1"/>
@@ -464,26 +464,26 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="49" fontId="2" fillId="2" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="49" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -916,127 +916,127 @@
   <sheetData>
     <row r="1" spans="2:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15" t="s">
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="J2" s="15"/>
-      <c r="K2" s="15"/>
-      <c r="L2" s="15"/>
-      <c r="M2" s="15"/>
+      <c r="J2" s="19"/>
+      <c r="K2" s="19"/>
+      <c r="L2" s="19"/>
+      <c r="M2" s="19"/>
     </row>
     <row r="3" spans="2:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="16" t="s">
+      <c r="B3" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
-      <c r="G3" s="16"/>
-      <c r="H3" s="16"/>
-      <c r="I3" s="17" t="s">
+      <c r="C3" s="17"/>
+      <c r="D3" s="17"/>
+      <c r="E3" s="17"/>
+      <c r="F3" s="17"/>
+      <c r="G3" s="17"/>
+      <c r="H3" s="17"/>
+      <c r="I3" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="J3" s="17"/>
-      <c r="K3" s="17"/>
-      <c r="L3" s="17"/>
-      <c r="M3" s="17"/>
+      <c r="J3" s="18"/>
+      <c r="K3" s="18"/>
+      <c r="L3" s="18"/>
+      <c r="M3" s="18"/>
     </row>
     <row r="4" spans="2:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="16"/>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="16"/>
-      <c r="G4" s="16"/>
-      <c r="H4" s="16"/>
-      <c r="I4" s="17" t="s">
+      <c r="C4" s="17"/>
+      <c r="D4" s="17"/>
+      <c r="E4" s="17"/>
+      <c r="F4" s="17"/>
+      <c r="G4" s="17"/>
+      <c r="H4" s="17"/>
+      <c r="I4" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="J4" s="17"/>
-      <c r="K4" s="17"/>
-      <c r="L4" s="17"/>
-      <c r="M4" s="17"/>
+      <c r="J4" s="18"/>
+      <c r="K4" s="18"/>
+      <c r="L4" s="18"/>
+      <c r="M4" s="18"/>
     </row>
     <row r="5" spans="2:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="16"/>
-      <c r="D5" s="16"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="16"/>
-      <c r="G5" s="16"/>
-      <c r="H5" s="16"/>
-      <c r="I5" s="17" t="s">
+      <c r="C5" s="17"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="17"/>
+      <c r="F5" s="17"/>
+      <c r="G5" s="17"/>
+      <c r="H5" s="17"/>
+      <c r="I5" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="J5" s="17"/>
-      <c r="K5" s="17"/>
-      <c r="L5" s="17"/>
-      <c r="M5" s="17"/>
+      <c r="J5" s="18"/>
+      <c r="K5" s="18"/>
+      <c r="L5" s="18"/>
+      <c r="M5" s="18"/>
     </row>
     <row r="6" spans="2:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="16"/>
-      <c r="F6" s="16"/>
-      <c r="G6" s="16"/>
-      <c r="H6" s="16"/>
-      <c r="I6" s="17" t="s">
+      <c r="C6" s="17"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="17"/>
+      <c r="I6" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="J6" s="17"/>
-      <c r="K6" s="17"/>
-      <c r="L6" s="17"/>
-      <c r="M6" s="17"/>
+      <c r="J6" s="18"/>
+      <c r="K6" s="18"/>
+      <c r="L6" s="18"/>
+      <c r="M6" s="18"/>
     </row>
     <row r="7" spans="2:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="8" spans="2:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="18"/>
-      <c r="D8" s="18"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
-      <c r="G8" s="18"/>
-      <c r="H8" s="18"/>
-      <c r="I8" s="18"/>
-      <c r="J8" s="18"/>
-      <c r="K8" s="18"/>
-      <c r="L8" s="18"/>
-      <c r="M8" s="18"/>
+      <c r="C8" s="20"/>
+      <c r="D8" s="20"/>
+      <c r="E8" s="20"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="20"/>
+      <c r="H8" s="20"/>
+      <c r="I8" s="20"/>
+      <c r="J8" s="20"/>
+      <c r="K8" s="20"/>
+      <c r="L8" s="20"/>
+      <c r="M8" s="20"/>
     </row>
     <row r="9" spans="2:26" ht="112.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="19"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="19"/>
-      <c r="F9" s="19"/>
-      <c r="G9" s="19"/>
-      <c r="H9" s="19"/>
-      <c r="I9" s="19"/>
-      <c r="J9" s="19"/>
-      <c r="K9" s="19"/>
-      <c r="L9" s="19"/>
-      <c r="M9" s="19"/>
+      <c r="C9" s="21"/>
+      <c r="D9" s="21"/>
+      <c r="E9" s="21"/>
+      <c r="F9" s="21"/>
+      <c r="G9" s="21"/>
+      <c r="H9" s="21"/>
+      <c r="I9" s="21"/>
+      <c r="J9" s="21"/>
+      <c r="K9" s="21"/>
+      <c r="L9" s="21"/>
+      <c r="M9" s="21"/>
     </row>
     <row r="10" spans="2:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="4"/>
@@ -1058,29 +1058,29 @@
       </c>
     </row>
     <row r="12" spans="2:26" ht="16" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="20" t="s">
-        <v>13</v>
-      </c>
-      <c r="C12" s="20"/>
-      <c r="D12" s="20"/>
-      <c r="E12" s="20"/>
-      <c r="F12" s="20"/>
-      <c r="G12" s="20"/>
-      <c r="H12" s="20"/>
-      <c r="I12" s="20"/>
-      <c r="J12" s="20"/>
-      <c r="K12" s="20"/>
-      <c r="L12" s="20"/>
-      <c r="M12" s="20"/>
-      <c r="N12" s="20"/>
-      <c r="O12" s="20"/>
-      <c r="P12" s="20"/>
-      <c r="Q12" s="20"/>
-      <c r="R12" s="21" t="s">
+      <c r="B12" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="15"/>
+      <c r="H12" s="15"/>
+      <c r="I12" s="15"/>
+      <c r="J12" s="15"/>
+      <c r="K12" s="15"/>
+      <c r="L12" s="15"/>
+      <c r="M12" s="15"/>
+      <c r="N12" s="15"/>
+      <c r="O12" s="15"/>
+      <c r="P12" s="15"/>
+      <c r="Q12" s="15"/>
+      <c r="R12" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="S12" s="21"/>
-      <c r="T12" s="21"/>
+      <c r="S12" s="16"/>
+      <c r="T12" s="16"/>
       <c r="U12" s="5"/>
       <c r="V12" s="5"/>
       <c r="W12" s="5"/>
@@ -1279,6 +1279,11 @@
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
   <autoFilter ref="B13:Z15" xr:uid="{E9404A2D-0DA6-45EF-A78B-6224627D30F1}"/>
   <mergeCells count="13">
+    <mergeCell ref="B2:M2"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="I3:M3"/>
+    <mergeCell ref="B8:M8"/>
+    <mergeCell ref="B9:M9"/>
     <mergeCell ref="B12:Q12"/>
     <mergeCell ref="R12:T12"/>
     <mergeCell ref="B4:H4"/>
@@ -1287,11 +1292,6 @@
     <mergeCell ref="I5:M5"/>
     <mergeCell ref="B6:H6"/>
     <mergeCell ref="I6:M6"/>
-    <mergeCell ref="B2:M2"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="I3:M3"/>
-    <mergeCell ref="B8:M8"/>
-    <mergeCell ref="B9:M9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555551" footer="0.51180555555555551"/>
   <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -1320,127 +1320,127 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15" t="s">
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="J2" s="15"/>
-      <c r="K2" s="15"/>
-      <c r="L2" s="15"/>
-      <c r="M2" s="15"/>
+      <c r="J2" s="19"/>
+      <c r="K2" s="19"/>
+      <c r="L2" s="19"/>
+      <c r="M2" s="19"/>
     </row>
     <row r="3" spans="2:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="16" t="s">
+      <c r="B3" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
-      <c r="G3" s="16"/>
-      <c r="H3" s="16"/>
-      <c r="I3" s="17" t="s">
+      <c r="C3" s="17"/>
+      <c r="D3" s="17"/>
+      <c r="E3" s="17"/>
+      <c r="F3" s="17"/>
+      <c r="G3" s="17"/>
+      <c r="H3" s="17"/>
+      <c r="I3" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="J3" s="17"/>
-      <c r="K3" s="17"/>
-      <c r="L3" s="17"/>
-      <c r="M3" s="17"/>
+      <c r="J3" s="18"/>
+      <c r="K3" s="18"/>
+      <c r="L3" s="18"/>
+      <c r="M3" s="18"/>
     </row>
     <row r="4" spans="2:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="16"/>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="16"/>
-      <c r="G4" s="16"/>
-      <c r="H4" s="16"/>
-      <c r="I4" s="17" t="s">
+      <c r="C4" s="17"/>
+      <c r="D4" s="17"/>
+      <c r="E4" s="17"/>
+      <c r="F4" s="17"/>
+      <c r="G4" s="17"/>
+      <c r="H4" s="17"/>
+      <c r="I4" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="J4" s="17"/>
-      <c r="K4" s="17"/>
-      <c r="L4" s="17"/>
-      <c r="M4" s="17"/>
+      <c r="J4" s="18"/>
+      <c r="K4" s="18"/>
+      <c r="L4" s="18"/>
+      <c r="M4" s="18"/>
     </row>
     <row r="5" spans="2:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="16"/>
-      <c r="D5" s="16"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="16"/>
-      <c r="G5" s="16"/>
-      <c r="H5" s="16"/>
-      <c r="I5" s="17" t="s">
+      <c r="C5" s="17"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="17"/>
+      <c r="F5" s="17"/>
+      <c r="G5" s="17"/>
+      <c r="H5" s="17"/>
+      <c r="I5" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="J5" s="17"/>
-      <c r="K5" s="17"/>
-      <c r="L5" s="17"/>
-      <c r="M5" s="17"/>
+      <c r="J5" s="18"/>
+      <c r="K5" s="18"/>
+      <c r="L5" s="18"/>
+      <c r="M5" s="18"/>
     </row>
     <row r="6" spans="2:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="16"/>
-      <c r="F6" s="16"/>
-      <c r="G6" s="16"/>
-      <c r="H6" s="16"/>
-      <c r="I6" s="17" t="s">
+      <c r="C6" s="17"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="17"/>
+      <c r="I6" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="J6" s="17"/>
-      <c r="K6" s="17"/>
-      <c r="L6" s="17"/>
-      <c r="M6" s="17"/>
+      <c r="J6" s="18"/>
+      <c r="K6" s="18"/>
+      <c r="L6" s="18"/>
+      <c r="M6" s="18"/>
     </row>
     <row r="7" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="8" spans="2:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="18"/>
-      <c r="D8" s="18"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
-      <c r="G8" s="18"/>
-      <c r="H8" s="18"/>
-      <c r="I8" s="18"/>
-      <c r="J8" s="18"/>
-      <c r="K8" s="18"/>
-      <c r="L8" s="18"/>
-      <c r="M8" s="18"/>
+      <c r="C8" s="20"/>
+      <c r="D8" s="20"/>
+      <c r="E8" s="20"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="20"/>
+      <c r="H8" s="20"/>
+      <c r="I8" s="20"/>
+      <c r="J8" s="20"/>
+      <c r="K8" s="20"/>
+      <c r="L8" s="20"/>
+      <c r="M8" s="20"/>
     </row>
     <row r="9" spans="2:16" ht="144" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="C9" s="19"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="19"/>
-      <c r="F9" s="19"/>
-      <c r="G9" s="19"/>
-      <c r="H9" s="19"/>
-      <c r="I9" s="19"/>
-      <c r="J9" s="19"/>
-      <c r="K9" s="19"/>
-      <c r="L9" s="19"/>
-      <c r="M9" s="19"/>
+      <c r="C9" s="21"/>
+      <c r="D9" s="21"/>
+      <c r="E9" s="21"/>
+      <c r="F9" s="21"/>
+      <c r="G9" s="21"/>
+      <c r="H9" s="21"/>
+      <c r="I9" s="21"/>
+      <c r="J9" s="21"/>
+      <c r="K9" s="21"/>
+      <c r="L9" s="21"/>
+      <c r="M9" s="21"/>
     </row>
     <row r="10" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="12" spans="2:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">

</xml_diff>